<commit_message>
docs: populate all durations, start dates, and finish dates for HSU project tasks in Plan.xlsx
</commit_message>
<xml_diff>
--- a/Ebooks/Plan.xlsx
+++ b/Ebooks/Plan.xlsx
@@ -1117,9 +1117,18 @@
       <c r="B10" s="2" t="s">
         <v>15</v>
       </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="1"/>
+      <c r="C10" s="12">
+        <f>E10-D10</f>
+        <v>4</v>
+      </c>
+      <c r="D10" s="10">
+        <f>MIN(D11:D13)</f>
+        <v>46215</v>
+      </c>
+      <c r="E10" s="10">
+        <f>MAX(E11:E13)</f>
+        <v>46219</v>
+      </c>
       <c r="F10" s="1"/>
       <c r="G10" s="1"/>
       <c r="H10" s="1"/>
@@ -1158,9 +1167,16 @@
       <c r="B11" s="1" t="s">
         <v>23</v>
       </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="1"/>
-      <c r="E11" s="1"/>
+      <c r="C11" s="15">
+        <v>1</v>
+      </c>
+      <c r="D11" s="7">
+        <v>46215</v>
+      </c>
+      <c r="E11" s="7">
+        <f>D11+C11</f>
+        <v>46216</v>
+      </c>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
       <c r="H11" s="1"/>
@@ -1199,9 +1215,16 @@
       <c r="B12" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="C12" s="15"/>
-      <c r="D12" s="1"/>
-      <c r="E12" s="1"/>
+      <c r="C12" s="15">
+        <v>2</v>
+      </c>
+      <c r="D12" s="7">
+        <v>46216</v>
+      </c>
+      <c r="E12" s="7">
+        <f>D12+C12</f>
+        <v>46218</v>
+      </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
       <c r="H12" s="1"/>
@@ -1240,9 +1263,16 @@
       <c r="B13" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C13" s="15"/>
-      <c r="D13" s="1"/>
-      <c r="E13" s="1"/>
+      <c r="C13" s="15">
+        <v>1</v>
+      </c>
+      <c r="D13" s="7">
+        <v>46218</v>
+      </c>
+      <c r="E13" s="7">
+        <f>D13+C13</f>
+        <v>46219</v>
+      </c>
       <c r="F13" s="6"/>
       <c r="G13" s="6"/>
       <c r="H13" s="6"/>
@@ -1281,9 +1311,16 @@
       <c r="B14" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="C14" s="15"/>
-      <c r="D14" s="1"/>
-      <c r="E14" s="1"/>
+      <c r="C14" s="15">
+        <v>5</v>
+      </c>
+      <c r="D14" s="7">
+        <v>46218</v>
+      </c>
+      <c r="E14" s="7">
+        <f>D14+C14</f>
+        <v>46223</v>
+      </c>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
       <c r="H14" s="1"/>
@@ -1322,9 +1359,18 @@
       <c r="B15" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="C15" s="15"/>
-      <c r="D15" s="1"/>
-      <c r="E15" s="1"/>
+      <c r="C15" s="12">
+        <f>E15-D15</f>
+        <v>27</v>
+      </c>
+      <c r="D15" s="10">
+        <f>MIN(D16:D23)</f>
+        <v>46223</v>
+      </c>
+      <c r="E15" s="10">
+        <f>MAX(E16:E23)</f>
+        <v>46250</v>
+      </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
       <c r="H15" s="1"/>
@@ -1363,9 +1409,16 @@
       <c r="B16" s="1" t="s">
         <v>28</v>
       </c>
-      <c r="C16" s="15"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="1"/>
+      <c r="C16" s="15">
+        <v>3</v>
+      </c>
+      <c r="D16" s="7">
+        <v>46223</v>
+      </c>
+      <c r="E16" s="7">
+        <f>D16+C16</f>
+        <v>46226</v>
+      </c>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
       <c r="H16" s="1"/>
@@ -1404,9 +1457,16 @@
       <c r="B17" s="1" t="s">
         <v>29</v>
       </c>
-      <c r="C17" s="15"/>
-      <c r="D17" s="1"/>
-      <c r="E17" s="1"/>
+      <c r="C17" s="15">
+        <v>2</v>
+      </c>
+      <c r="D17" s="7">
+        <v>46226</v>
+      </c>
+      <c r="E17" s="7">
+        <f>D17+C17</f>
+        <v>46228</v>
+      </c>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
       <c r="H17" s="1"/>
@@ -1445,9 +1505,16 @@
       <c r="B18" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="C18" s="15"/>
-      <c r="D18" s="1"/>
-      <c r="E18" s="1"/>
+      <c r="C18" s="15">
+        <v>4</v>
+      </c>
+      <c r="D18" s="7">
+        <v>46228</v>
+      </c>
+      <c r="E18" s="7">
+        <f>D18+C18</f>
+        <v>46232</v>
+      </c>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
       <c r="H18" s="1"/>
@@ -1486,9 +1553,16 @@
       <c r="B19" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="C19" s="15"/>
-      <c r="D19" s="1"/>
-      <c r="E19" s="1"/>
+      <c r="C19" s="15">
+        <v>5</v>
+      </c>
+      <c r="D19" s="7">
+        <v>46228</v>
+      </c>
+      <c r="E19" s="7">
+        <f>D19+C19</f>
+        <v>46233</v>
+      </c>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
       <c r="H19" s="1"/>
@@ -1527,9 +1601,16 @@
       <c r="B20" s="1" t="s">
         <v>32</v>
       </c>
-      <c r="C20" s="15"/>
-      <c r="D20" s="1"/>
-      <c r="E20" s="1"/>
+      <c r="C20" s="15">
+        <v>11</v>
+      </c>
+      <c r="D20" s="7">
+        <v>46233</v>
+      </c>
+      <c r="E20" s="7">
+        <f>D20+C20</f>
+        <v>46244</v>
+      </c>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
       <c r="H20" s="1"/>
@@ -1568,9 +1649,16 @@
       <c r="B21" s="1" t="s">
         <v>33</v>
       </c>
-      <c r="C21" s="15"/>
-      <c r="D21" s="1"/>
-      <c r="E21" s="1"/>
+      <c r="C21" s="15">
+        <v>4</v>
+      </c>
+      <c r="D21" s="7">
+        <v>46244</v>
+      </c>
+      <c r="E21" s="7">
+        <f>D21+C21</f>
+        <v>46248</v>
+      </c>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
       <c r="H21" s="1"/>
@@ -1609,9 +1697,16 @@
       <c r="B22" s="1" t="s">
         <v>34</v>
       </c>
-      <c r="C22" s="15"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="1"/>
+      <c r="C22" s="15">
+        <v>3</v>
+      </c>
+      <c r="D22" s="7">
+        <v>46245</v>
+      </c>
+      <c r="E22" s="7">
+        <f>D22+C22</f>
+        <v>46248</v>
+      </c>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
       <c r="H22" s="1"/>
@@ -1650,9 +1745,16 @@
       <c r="B23" s="1" t="s">
         <v>35</v>
       </c>
-      <c r="C23" s="15"/>
-      <c r="D23" s="1"/>
-      <c r="E23" s="1"/>
+      <c r="C23" s="15">
+        <v>2</v>
+      </c>
+      <c r="D23" s="7">
+        <v>46248</v>
+      </c>
+      <c r="E23" s="7">
+        <f>D23+C23</f>
+        <v>46250</v>
+      </c>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
       <c r="H23" s="1"/>
@@ -1691,9 +1793,16 @@
       <c r="B24" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="C24" s="15"/>
-      <c r="D24" s="1"/>
-      <c r="E24" s="1"/>
+      <c r="C24" s="15">
+        <v>35</v>
+      </c>
+      <c r="D24" s="7">
+        <v>46215</v>
+      </c>
+      <c r="E24" s="7">
+        <f>D24+C24</f>
+        <v>46250</v>
+      </c>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
       <c r="H24" s="1"/>
@@ -1732,9 +1841,16 @@
       <c r="B25" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="C25" s="15"/>
-      <c r="D25" s="1"/>
-      <c r="E25" s="1"/>
+      <c r="C25" s="15">
+        <v>3</v>
+      </c>
+      <c r="D25" s="7">
+        <v>46247</v>
+      </c>
+      <c r="E25" s="7">
+        <f>D25+C25</f>
+        <v>46250</v>
+      </c>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
       <c r="H25" s="1"/>

</xml_diff>

<commit_message>
fix(plan): replace MINIFS/MAXIFS with highly compatible INDEX/MATCH and LOOKUP formulas
</commit_message>
<xml_diff>
--- a/Ebooks/Plan.xlsx
+++ b/Ebooks/Plan.xlsx
@@ -1521,10 +1521,10 @@
         <f>COUNTIF(F5:CB5,"█")</f>
       </c>
       <c r="D5" s="11">
-        <f>IF(C5&gt;0,MINIFS(F$1:CB$1,F5:CB5,"█"),"")</f>
+        <f>IF(C5&gt;0,INDEX(F$1:CB$1,MATCH("█",F5:CB5,0)),"")</f>
       </c>
       <c r="E5" s="11">
-        <f>IF(C5&gt;0,MAXIFS(F$1:CB$1,F5:CB5,"█"),"")</f>
+        <f>IF(C5&gt;0,LOOKUP(2,1/(F5:CB5="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F5" s="2"/>
       <c r="G5" s="2"/>
@@ -1613,10 +1613,10 @@
         <f>COUNTIF(F6:CB6,"█")</f>
       </c>
       <c r="D6" s="11">
-        <f>IF(C6&gt;0,MINIFS(F$1:CB$1,F6:CB6,"█"),"")</f>
+        <f>IF(C6&gt;0,INDEX(F$1:CB$1,MATCH("█",F6:CB6,0)),"")</f>
       </c>
       <c r="E6" s="11">
-        <f>IF(C6&gt;0,MAXIFS(F$1:CB$1,F6:CB6,"█"),"")</f>
+        <f>IF(C6&gt;0,LOOKUP(2,1/(F6:CB6="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F6" s="2" t="s">
         <v>28</v>
@@ -1709,10 +1709,10 @@
         <f>COUNTIF(F7:CB7,"█")</f>
       </c>
       <c r="D7" s="11">
-        <f>IF(C7&gt;0,MINIFS(F$1:CB$1,F7:CB7,"█"),"")</f>
+        <f>IF(C7&gt;0,INDEX(F$1:CB$1,MATCH("█",F7:CB7,0)),"")</f>
       </c>
       <c r="E7" s="11">
-        <f>IF(C7&gt;0,MAXIFS(F$1:CB$1,F7:CB7,"█"),"")</f>
+        <f>IF(C7&gt;0,LOOKUP(2,1/(F7:CB7="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F7" s="2"/>
       <c r="G7" s="2"/>
@@ -1807,10 +1807,10 @@
         <f>COUNTIF(F8:CB8,"█")</f>
       </c>
       <c r="D8" s="11">
-        <f>IF(C8&gt;0,MINIFS(F$1:CB$1,F8:CB8,"█"),"")</f>
+        <f>IF(C8&gt;0,INDEX(F$1:CB$1,MATCH("█",F8:CB8,0)),"")</f>
       </c>
       <c r="E8" s="11">
-        <f>IF(C8&gt;0,MAXIFS(F$1:CB$1,F8:CB8,"█"),"")</f>
+        <f>IF(C8&gt;0,LOOKUP(2,1/(F8:CB8="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F8" s="2"/>
       <c r="G8" s="2"/>
@@ -1899,10 +1899,10 @@
         <f>COUNTIF(F9:CB9,"█")</f>
       </c>
       <c r="D9" s="11">
-        <f>IF(C9&gt;0,MINIFS(F$1:CB$1,F9:CB9,"█"),"")</f>
+        <f>IF(C9&gt;0,INDEX(F$1:CB$1,MATCH("█",F9:CB9,0)),"")</f>
       </c>
       <c r="E9" s="11">
-        <f>IF(C9&gt;0,MAXIFS(F$1:CB$1,F9:CB9,"█"),"")</f>
+        <f>IF(C9&gt;0,LOOKUP(2,1/(F9:CB9="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F9" s="2"/>
       <c r="G9" s="2"/>
@@ -2239,10 +2239,10 @@
         <f>COUNTIF(F11:CB11,"█")</f>
       </c>
       <c r="D11" s="11">
-        <f>IF(C11&gt;0,MINIFS(F$1:CB$1,F11:CB11,"█"),"")</f>
+        <f>IF(C11&gt;0,INDEX(F$1:CB$1,MATCH("█",F11:CB11,0)),"")</f>
       </c>
       <c r="E11" s="11">
-        <f>IF(C11&gt;0,MAXIFS(F$1:CB$1,F11:CB11,"█"),"")</f>
+        <f>IF(C11&gt;0,LOOKUP(2,1/(F11:CB11="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F11" s="2" t="s">
         <v>28</v>
@@ -2333,10 +2333,10 @@
         <f>COUNTIF(F12:CB12,"█")</f>
       </c>
       <c r="D12" s="11">
-        <f>IF(C12&gt;0,MINIFS(F$1:CB$1,F12:CB12,"█"),"")</f>
+        <f>IF(C12&gt;0,INDEX(F$1:CB$1,MATCH("█",F12:CB12,0)),"")</f>
       </c>
       <c r="E12" s="11">
-        <f>IF(C12&gt;0,MAXIFS(F$1:CB$1,F12:CB12,"█"),"")</f>
+        <f>IF(C12&gt;0,LOOKUP(2,1/(F12:CB12="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F12" s="2"/>
       <c r="G12" s="2" t="s">
@@ -2431,10 +2431,10 @@
         <f>COUNTIF(F13:CB13,"█")</f>
       </c>
       <c r="D13" s="11">
-        <f>IF(C13&gt;0,MINIFS(F$1:CB$1,F13:CB13,"█"),"")</f>
+        <f>IF(C13&gt;0,INDEX(F$1:CB$1,MATCH("█",F13:CB13,0)),"")</f>
       </c>
       <c r="E13" s="11">
-        <f>IF(C13&gt;0,MAXIFS(F$1:CB$1,F13:CB13,"█"),"")</f>
+        <f>IF(C13&gt;0,LOOKUP(2,1/(F13:CB13="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F13" s="2"/>
       <c r="G13" s="2"/>
@@ -2525,10 +2525,10 @@
         <f>COUNTIF(F14:CB14,"█")</f>
       </c>
       <c r="D14" s="11">
-        <f>IF(C14&gt;0,MINIFS(F$1:CB$1,F14:CB14,"█"),"")</f>
+        <f>IF(C14&gt;0,INDEX(F$1:CB$1,MATCH("█",F14:CB14,0)),"")</f>
       </c>
       <c r="E14" s="11">
-        <f>IF(C14&gt;0,MAXIFS(F$1:CB$1,F14:CB14,"█"),"")</f>
+        <f>IF(C14&gt;0,LOOKUP(2,1/(F14:CB14="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F14" s="2" t="s">
         <v>28</v>
@@ -2883,10 +2883,10 @@
         <f>COUNTIF(F16:CB16,"█")</f>
       </c>
       <c r="D16" s="11">
-        <f>IF(C16&gt;0,MINIFS(F$1:CB$1,F16:CB16,"█"),"")</f>
+        <f>IF(C16&gt;0,INDEX(F$1:CB$1,MATCH("█",F16:CB16,0)),"")</f>
       </c>
       <c r="E16" s="11">
-        <f>IF(C16&gt;0,MAXIFS(F$1:CB$1,F16:CB16,"█"),"")</f>
+        <f>IF(C16&gt;0,LOOKUP(2,1/(F16:CB16="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F16" s="2"/>
       <c r="G16" s="2"/>
@@ -2979,10 +2979,10 @@
         <f>COUNTIF(F17:CB17,"█")</f>
       </c>
       <c r="D17" s="11">
-        <f>IF(C17&gt;0,MINIFS(F$1:CB$1,F17:CB17,"█"),"")</f>
+        <f>IF(C17&gt;0,INDEX(F$1:CB$1,MATCH("█",F17:CB17,0)),"")</f>
       </c>
       <c r="E17" s="11">
-        <f>IF(C17&gt;0,MAXIFS(F$1:CB$1,F17:CB17,"█"),"")</f>
+        <f>IF(C17&gt;0,LOOKUP(2,1/(F17:CB17="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F17" s="2"/>
       <c r="G17" s="2"/>
@@ -3077,10 +3077,10 @@
         <f>COUNTIF(F18:CB18,"█")</f>
       </c>
       <c r="D18" s="11">
-        <f>IF(C18&gt;0,MINIFS(F$1:CB$1,F18:CB18,"█"),"")</f>
+        <f>IF(C18&gt;0,INDEX(F$1:CB$1,MATCH("█",F18:CB18,0)),"")</f>
       </c>
       <c r="E18" s="11">
-        <f>IF(C18&gt;0,MAXIFS(F$1:CB$1,F18:CB18,"█"),"")</f>
+        <f>IF(C18&gt;0,LOOKUP(2,1/(F18:CB18="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F18" s="2"/>
       <c r="G18" s="2"/>
@@ -3175,10 +3175,10 @@
         <f>COUNTIF(F19:CB19,"█")</f>
       </c>
       <c r="D19" s="11">
-        <f>IF(C19&gt;0,MINIFS(F$1:CB$1,F19:CB19,"█"),"")</f>
+        <f>IF(C19&gt;0,INDEX(F$1:CB$1,MATCH("█",F19:CB19,0)),"")</f>
       </c>
       <c r="E19" s="11">
-        <f>IF(C19&gt;0,MAXIFS(F$1:CB$1,F19:CB19,"█"),"")</f>
+        <f>IF(C19&gt;0,LOOKUP(2,1/(F19:CB19="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F19" s="2"/>
       <c r="G19" s="2"/>
@@ -3275,10 +3275,10 @@
         <f>COUNTIF(F20:CB20,"█")</f>
       </c>
       <c r="D20" s="11">
-        <f>IF(C20&gt;0,MINIFS(F$1:CB$1,F20:CB20,"█"),"")</f>
+        <f>IF(C20&gt;0,INDEX(F$1:CB$1,MATCH("█",F20:CB20,0)),"")</f>
       </c>
       <c r="E20" s="11">
-        <f>IF(C20&gt;0,MAXIFS(F$1:CB$1,F20:CB20,"█"),"")</f>
+        <f>IF(C20&gt;0,LOOKUP(2,1/(F20:CB20="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F20" s="2"/>
       <c r="G20" s="2"/>
@@ -3383,10 +3383,10 @@
         <f>COUNTIF(F21:CB21,"█")</f>
       </c>
       <c r="D21" s="11">
-        <f>IF(C21&gt;0,MINIFS(F$1:CB$1,F21:CB21,"█"),"")</f>
+        <f>IF(C21&gt;0,INDEX(F$1:CB$1,MATCH("█",F21:CB21,0)),"")</f>
       </c>
       <c r="E21" s="11">
-        <f>IF(C21&gt;0,MAXIFS(F$1:CB$1,F21:CB21,"█"),"")</f>
+        <f>IF(C21&gt;0,LOOKUP(2,1/(F21:CB21="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -3481,10 +3481,10 @@
         <f>COUNTIF(F22:CB22,"█")</f>
       </c>
       <c r="D22" s="11">
-        <f>IF(C22&gt;0,MINIFS(F$1:CB$1,F22:CB22,"█"),"")</f>
+        <f>IF(C22&gt;0,INDEX(F$1:CB$1,MATCH("█",F22:CB22,0)),"")</f>
       </c>
       <c r="E22" s="11">
-        <f>IF(C22&gt;0,MAXIFS(F$1:CB$1,F22:CB22,"█"),"")</f>
+        <f>IF(C22&gt;0,LOOKUP(2,1/(F22:CB22="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -3581,10 +3581,10 @@
         <f>COUNTIF(F23:CB23,"█")</f>
       </c>
       <c r="D23" s="11">
-        <f>IF(C23&gt;0,MINIFS(F$1:CB$1,F23:CB23,"█"),"")</f>
+        <f>IF(C23&gt;0,INDEX(F$1:CB$1,MATCH("█",F23:CB23,0)),"")</f>
       </c>
       <c r="E23" s="11">
-        <f>IF(C23&gt;0,MAXIFS(F$1:CB$1,F23:CB23,"█"),"")</f>
+        <f>IF(C23&gt;0,LOOKUP(2,1/(F23:CB23="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -3675,10 +3675,10 @@
         <f>COUNTIF(F24:CB24,"█")</f>
       </c>
       <c r="D24" s="11">
-        <f>IF(C24&gt;0,MINIFS(F$1:CB$1,F24:CB24,"█"),"")</f>
+        <f>IF(C24&gt;0,INDEX(F$1:CB$1,MATCH("█",F24:CB24,0)),"")</f>
       </c>
       <c r="E24" s="11">
-        <f>IF(C24&gt;0,MAXIFS(F$1:CB$1,F24:CB24,"█"),"")</f>
+        <f>IF(C24&gt;0,LOOKUP(2,1/(F24:CB24="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F24" s="2" t="s">
         <v>28</v>
@@ -3817,10 +3817,10 @@
         <f>COUNTIF(F25:CB25,"█")</f>
       </c>
       <c r="D25" s="11">
-        <f>IF(C25&gt;0,MINIFS(F$1:CB$1,F25:CB25,"█"),"")</f>
+        <f>IF(C25&gt;0,INDEX(F$1:CB$1,MATCH("█",F25:CB25,0)),"")</f>
       </c>
       <c r="E25" s="11">
-        <f>IF(C25&gt;0,MAXIFS(F$1:CB$1,F25:CB25,"█"),"")</f>
+        <f>IF(C25&gt;0,LOOKUP(2,1/(F25:CB25="█"),F$1:CB$1),"")</f>
       </c>
       <c r="F25" s="2"/>
       <c r="G25" s="2"/>

</xml_diff>

<commit_message>
feat(plan): populate exact project schedule baseline gantt colors into Plan.xlsx
</commit_message>
<xml_diff>
--- a/Ebooks/Plan.xlsx
+++ b/Ebooks/Plan.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="136" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="48">
   <si>
     <t>WBS</t>
   </si>
@@ -1529,7 +1529,9 @@
       <c r="F5" s="2" t="s">
         <v>27</v>
       </c>
-      <c r="G5" s="2"/>
+      <c r="G5" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="H5" s="2"/>
       <c r="I5" s="2"/>
       <c r="J5" s="2"/>
@@ -1620,11 +1622,11 @@
       <c r="E6" s="11">
         <f>IF(C6&gt;0,INDEX(F$1:CB$1,MATCH("█",F6:CB6,0)+C6-1),"")</f>
       </c>
-      <c r="F6" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F6" s="2"/>
       <c r="G6" s="2"/>
-      <c r="H6" s="2"/>
+      <c r="H6" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="I6" s="2"/>
       <c r="J6" s="2"/>
       <c r="K6" s="2"/>
@@ -1714,13 +1716,15 @@
       <c r="E7" s="11">
         <f>IF(C7&gt;0,INDEX(F$1:CB$1,MATCH("█",F7:CB7,0)+C7-1),"")</f>
       </c>
-      <c r="F7" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F7" s="2"/>
       <c r="G7" s="2"/>
       <c r="H7" s="2"/>
-      <c r="I7" s="2"/>
-      <c r="J7" s="2"/>
+      <c r="I7" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J7" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="K7" s="2"/>
       <c r="L7" s="2"/>
       <c r="M7" s="2"/>
@@ -1808,14 +1812,14 @@
       <c r="E8" s="11">
         <f>IF(C8&gt;0,INDEX(F$1:CB$1,MATCH("█",F8:CB8,0)+C8-1),"")</f>
       </c>
-      <c r="F8" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F8" s="2"/>
       <c r="G8" s="2"/>
       <c r="H8" s="2"/>
       <c r="I8" s="2"/>
       <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
+      <c r="K8" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="L8" s="2"/>
       <c r="M8" s="2"/>
       <c r="N8" s="2"/>
@@ -1902,14 +1906,18 @@
       <c r="E9" s="11">
         <f>IF(C9&gt;0,INDEX(F$1:CB$1,MATCH("█",F9:CB9,0)+C9-1),"")</f>
       </c>
-      <c r="F9" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F9" s="2"/>
       <c r="G9" s="2"/>
       <c r="H9" s="2"/>
-      <c r="I9" s="2"/>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
+      <c r="I9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="J9" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="K9" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="L9" s="2"/>
       <c r="M9" s="2"/>
       <c r="N9" s="2"/>
@@ -2238,15 +2246,15 @@
       <c r="E11" s="11">
         <f>IF(C11&gt;0,INDEX(F$1:CB$1,MATCH("█",F11:CB11,0)+C11-1),"")</f>
       </c>
-      <c r="F11" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F11" s="2"/>
       <c r="G11" s="2"/>
       <c r="H11" s="2"/>
       <c r="I11" s="2"/>
       <c r="J11" s="2"/>
       <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
+      <c r="L11" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="M11" s="2"/>
       <c r="N11" s="2"/>
       <c r="O11" s="2"/>
@@ -2332,17 +2340,19 @@
       <c r="E12" s="11">
         <f>IF(C12&gt;0,INDEX(F$1:CB$1,MATCH("█",F12:CB12,0)+C12-1),"")</f>
       </c>
-      <c r="F12" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F12" s="2"/>
       <c r="G12" s="2"/>
       <c r="H12" s="2"/>
       <c r="I12" s="2"/>
       <c r="J12" s="2"/>
       <c r="K12" s="2"/>
       <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
-      <c r="N12" s="2"/>
+      <c r="M12" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N12" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="O12" s="2"/>
       <c r="P12" s="2"/>
       <c r="Q12" s="2"/>
@@ -2426,9 +2436,7 @@
       <c r="E13" s="11">
         <f>IF(C13&gt;0,INDEX(F$1:CB$1,MATCH("█",F13:CB13,0)+C13-1),"")</f>
       </c>
-      <c r="F13" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F13" s="2"/>
       <c r="G13" s="2"/>
       <c r="H13" s="2"/>
       <c r="I13" s="2"/>
@@ -2437,7 +2445,9 @@
       <c r="L13" s="2"/>
       <c r="M13" s="2"/>
       <c r="N13" s="2"/>
-      <c r="O13" s="2"/>
+      <c r="O13" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="P13" s="2"/>
       <c r="Q13" s="2"/>
       <c r="R13" s="2"/>
@@ -2520,9 +2530,7 @@
       <c r="E14" s="11">
         <f>IF(C14&gt;0,INDEX(F$1:CB$1,MATCH("█",F14:CB14,0)+C14-1),"")</f>
       </c>
-      <c r="F14" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F14" s="2"/>
       <c r="G14" s="2"/>
       <c r="H14" s="2"/>
       <c r="I14" s="2"/>
@@ -2532,11 +2540,21 @@
       <c r="M14" s="2"/>
       <c r="N14" s="2"/>
       <c r="O14" s="2"/>
-      <c r="P14" s="2"/>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="2"/>
+      <c r="P14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T14" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="U14" s="2"/>
       <c r="V14" s="2"/>
       <c r="W14" s="2"/>
@@ -2856,9 +2874,7 @@
       <c r="E16" s="11">
         <f>IF(C16&gt;0,INDEX(F$1:CB$1,MATCH("█",F16:CB16,0)+C16-1),"")</f>
       </c>
-      <c r="F16" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F16" s="2"/>
       <c r="G16" s="2"/>
       <c r="H16" s="2"/>
       <c r="I16" s="2"/>
@@ -2873,9 +2889,15 @@
       <c r="R16" s="2"/>
       <c r="S16" s="2"/>
       <c r="T16" s="2"/>
-      <c r="U16" s="2"/>
-      <c r="V16" s="2"/>
-      <c r="W16" s="2"/>
+      <c r="U16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V16" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W16" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="X16" s="2"/>
       <c r="Y16" s="2"/>
       <c r="Z16" s="2"/>
@@ -2950,9 +2972,7 @@
       <c r="E17" s="11">
         <f>IF(C17&gt;0,INDEX(F$1:CB$1,MATCH("█",F17:CB17,0)+C17-1),"")</f>
       </c>
-      <c r="F17" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F17" s="2"/>
       <c r="G17" s="2"/>
       <c r="H17" s="2"/>
       <c r="I17" s="2"/>
@@ -2970,8 +2990,12 @@
       <c r="U17" s="2"/>
       <c r="V17" s="2"/>
       <c r="W17" s="2"/>
-      <c r="X17" s="2"/>
-      <c r="Y17" s="2"/>
+      <c r="X17" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y17" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="Z17" s="2"/>
       <c r="AA17" s="2"/>
       <c r="AB17" s="2"/>
@@ -3044,9 +3068,7 @@
       <c r="E18" s="11">
         <f>IF(C18&gt;0,INDEX(F$1:CB$1,MATCH("█",F18:CB18,0)+C18-1),"")</f>
       </c>
-      <c r="F18" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F18" s="2"/>
       <c r="G18" s="2"/>
       <c r="H18" s="2"/>
       <c r="I18" s="2"/>
@@ -3066,10 +3088,18 @@
       <c r="W18" s="2"/>
       <c r="X18" s="2"/>
       <c r="Y18" s="2"/>
-      <c r="Z18" s="2"/>
-      <c r="AA18" s="2"/>
-      <c r="AB18" s="2"/>
-      <c r="AC18" s="2"/>
+      <c r="Z18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB18" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC18" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="AD18" s="2"/>
       <c r="AE18" s="2"/>
       <c r="AF18" s="2"/>
@@ -3138,9 +3168,7 @@
       <c r="E19" s="11">
         <f>IF(C19&gt;0,INDEX(F$1:CB$1,MATCH("█",F19:CB19,0)+C19-1),"")</f>
       </c>
-      <c r="F19" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F19" s="2"/>
       <c r="G19" s="2"/>
       <c r="H19" s="2"/>
       <c r="I19" s="2"/>
@@ -3160,11 +3188,21 @@
       <c r="W19" s="2"/>
       <c r="X19" s="2"/>
       <c r="Y19" s="2"/>
-      <c r="Z19" s="2"/>
-      <c r="AA19" s="2"/>
-      <c r="AB19" s="2"/>
-      <c r="AC19" s="2"/>
-      <c r="AD19" s="2"/>
+      <c r="Z19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC19" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD19" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="AE19" s="2"/>
       <c r="AF19" s="2"/>
       <c r="AG19" s="2"/>
@@ -3232,9 +3270,7 @@
       <c r="E20" s="11">
         <f>IF(C20&gt;0,INDEX(F$1:CB$1,MATCH("█",F20:CB20,0)+C20-1),"")</f>
       </c>
-      <c r="F20" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F20" s="2"/>
       <c r="G20" s="2"/>
       <c r="H20" s="2"/>
       <c r="I20" s="2"/>
@@ -3259,17 +3295,39 @@
       <c r="AB20" s="2"/>
       <c r="AC20" s="2"/>
       <c r="AD20" s="2"/>
-      <c r="AE20" s="2"/>
-      <c r="AF20" s="2"/>
-      <c r="AG20" s="2"/>
-      <c r="AH20" s="2"/>
-      <c r="AI20" s="2"/>
-      <c r="AJ20" s="2"/>
-      <c r="AK20" s="2"/>
-      <c r="AL20" s="2"/>
-      <c r="AM20" s="2"/>
-      <c r="AN20" s="2"/>
-      <c r="AO20" s="2"/>
+      <c r="AE20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AF20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AG20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AH20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AI20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AJ20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AK20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AL20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AM20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AN20" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AO20" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="AP20" s="2"/>
       <c r="AQ20" s="2"/>
       <c r="AR20" s="2"/>
@@ -3326,9 +3384,7 @@
       <c r="E21" s="11">
         <f>IF(C21&gt;0,INDEX(F$1:CB$1,MATCH("█",F21:CB21,0)+C21-1),"")</f>
       </c>
-      <c r="F21" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F21" s="2"/>
       <c r="G21" s="2"/>
       <c r="H21" s="2"/>
       <c r="I21" s="2"/>
@@ -3364,10 +3420,18 @@
       <c r="AM21" s="2"/>
       <c r="AN21" s="2"/>
       <c r="AO21" s="2"/>
-      <c r="AP21" s="2"/>
-      <c r="AQ21" s="2"/>
-      <c r="AR21" s="2"/>
-      <c r="AS21" s="2"/>
+      <c r="AP21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AQ21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AR21" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AS21" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="AT21" s="2"/>
       <c r="AU21" s="2"/>
       <c r="AV21" s="2"/>
@@ -3420,9 +3484,7 @@
       <c r="E22" s="11">
         <f>IF(C22&gt;0,INDEX(F$1:CB$1,MATCH("█",F22:CB22,0)+C22-1),"")</f>
       </c>
-      <c r="F22" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F22" s="2"/>
       <c r="G22" s="2"/>
       <c r="H22" s="2"/>
       <c r="I22" s="2"/>
@@ -3462,9 +3524,15 @@
       <c r="AQ22" s="2"/>
       <c r="AR22" s="2"/>
       <c r="AS22" s="2"/>
-      <c r="AT22" s="2"/>
-      <c r="AU22" s="2"/>
-      <c r="AV22" s="2"/>
+      <c r="AT22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AU22" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AV22" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="AW22" s="2"/>
       <c r="AX22" s="2"/>
       <c r="AY22" s="2"/>
@@ -3514,9 +3582,7 @@
       <c r="E23" s="11">
         <f>IF(C23&gt;0,INDEX(F$1:CB$1,MATCH("█",F23:CB23,0)+C23-1),"")</f>
       </c>
-      <c r="F23" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F23" s="2"/>
       <c r="G23" s="2"/>
       <c r="H23" s="2"/>
       <c r="I23" s="2"/>
@@ -3559,8 +3625,12 @@
       <c r="AT23" s="2"/>
       <c r="AU23" s="2"/>
       <c r="AV23" s="2"/>
-      <c r="AW23" s="2"/>
-      <c r="AX23" s="2"/>
+      <c r="AW23" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AX23" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="AY23" s="2"/>
       <c r="AZ23" s="2"/>
       <c r="BA23" s="2"/>
@@ -3608,49 +3678,117 @@
       <c r="E24" s="11">
         <f>IF(C24&gt;0,INDEX(F$1:CB$1,MATCH("█",F24:CB24,0)+C24-1),"")</f>
       </c>
-      <c r="F24" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F24" s="2"/>
       <c r="G24" s="2"/>
       <c r="H24" s="2"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
-      <c r="L24" s="2"/>
-      <c r="M24" s="2"/>
-      <c r="N24" s="2"/>
-      <c r="O24" s="2"/>
-      <c r="P24" s="2"/>
-      <c r="Q24" s="2"/>
-      <c r="R24" s="2"/>
-      <c r="S24" s="2"/>
-      <c r="T24" s="2"/>
-      <c r="U24" s="2"/>
-      <c r="V24" s="2"/>
-      <c r="W24" s="2"/>
-      <c r="X24" s="2"/>
-      <c r="Y24" s="2"/>
-      <c r="Z24" s="2"/>
-      <c r="AA24" s="2"/>
-      <c r="AB24" s="2"/>
-      <c r="AC24" s="2"/>
-      <c r="AD24" s="2"/>
-      <c r="AE24" s="2"/>
-      <c r="AF24" s="2"/>
-      <c r="AG24" s="2"/>
-      <c r="AH24" s="2"/>
-      <c r="AI24" s="2"/>
-      <c r="AJ24" s="2"/>
-      <c r="AK24" s="2"/>
-      <c r="AL24" s="2"/>
-      <c r="AM24" s="2"/>
-      <c r="AN24" s="2"/>
-      <c r="AO24" s="2"/>
-      <c r="AP24" s="2"/>
-      <c r="AQ24" s="2"/>
-      <c r="AR24" s="2"/>
-      <c r="AS24" s="2"/>
-      <c r="AT24" s="2"/>
+      <c r="L24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="M24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="N24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="O24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="P24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Q24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="R24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="S24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="T24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="U24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="V24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="W24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="X24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Y24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AA24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AB24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AC24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AD24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AE24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AF24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AG24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AH24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AI24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AJ24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AK24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AL24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AM24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AN24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AO24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AP24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AQ24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AR24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AS24" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AT24" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="AU24" s="2"/>
       <c r="AV24" s="2"/>
       <c r="AW24" s="2"/>
@@ -3702,9 +3840,7 @@
       <c r="E25" s="11">
         <f>IF(C25&gt;0,INDEX(F$1:CB$1,MATCH("█",F25:CB25,0)+C25-1),"")</f>
       </c>
-      <c r="F25" s="2" t="s">
-        <v>27</v>
-      </c>
+      <c r="F25" s="2"/>
       <c r="G25" s="2"/>
       <c r="H25" s="2"/>
       <c r="I25" s="2"/>
@@ -3749,9 +3885,15 @@
       <c r="AV25" s="2"/>
       <c r="AW25" s="2"/>
       <c r="AX25" s="2"/>
-      <c r="AY25" s="2"/>
-      <c r="AZ25" s="2"/>
-      <c r="BA25" s="2"/>
+      <c r="AY25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="AZ25" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="BA25" s="2" t="s">
+        <v>27</v>
+      </c>
       <c r="BB25" s="2"/>
       <c r="BC25" s="2"/>
       <c r="BD25" s="2"/>

</xml_diff>